<commit_message>
fix: actualizar SHAs de trazabilidad tras rebase con origin/main
</commit_message>
<xml_diff>
--- a/docs/03_implementacion/MATRIZ-DOBLE-ENTRADA-SGMI.xlsx
+++ b/docs/03_implementacion/MATRIZ-DOBLE-ENTRADA-SGMI.xlsx
@@ -429,7 +429,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generado: 2026-07-03 00:23</t>
+          <t>Generado: 2026-07-03 00:39</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3a86b19</t>
+          <t>04c5fef</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>c87eb90</t>
+          <t>8836ddb</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>7d45f96</t>
+          <t>7814d12</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>bae1be7</t>
+          <t>1fde769</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>c54af96</t>
+          <t>f8e9e43</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ca8984c</t>
+          <t>1846117</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>aef66a6</t>
+          <t>9406618</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>af753d9</t>
+          <t>b6affb4</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2d8efad</t>
+          <t>4568914</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>21221d4</t>
+          <t>ac826f7</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>af7ce42</t>
+          <t>251f9a5</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>61832f7</t>
+          <t>ea3e62a</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0cfae15</t>
+          <t>7b17b7b</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>a77b6bb</t>
+          <t>c0a0952</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>f96c2f6</t>
+          <t>ce43d09</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1f2f8ce</t>
+          <t>1f31467</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>6924a69</t>
+          <t>09b175e</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>65a0cb3</t>
+          <t>3310b73</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>425c4fe</t>
+          <t>b185b2d</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>dc3da3e</t>
+          <t>60767bd</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>6ef1cdd</t>
+          <t>db3e558</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>7c6a056</t>
+          <t>086a1e5</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>7677c89</t>
+          <t>54960ad</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>201a1c8</t>
+          <t>1bc52f7</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>636635d</t>
+          <t>e99962c</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>c843789</t>
+          <t>46426ab</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>commit 3a86b19 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
+          <t>commit 04c5fef | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>commit c87eb90 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
+          <t>commit 8836ddb | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>commit 7d45f96 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
+          <t>commit 7814d12 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>commit bae1be7 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
+          <t>commit 1fde769 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>commit c54af96 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
+          <t>commit f8e9e43 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>commit ca8984c | impl 5a891bd | prompts/01_requisitos/R-002_historias_usuario_v1.md</t>
+          <t>commit 1846117 | impl 5a891bd | prompts/01_requisitos/R-002_historias_usuario_v1.md</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2459,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>commit aef66a6 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
+          <t>commit 9406618 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>commit af753d9 | impl 5a891bd | prompts/01_requisitos/R-002_historias_usuario_v1.md</t>
+          <t>commit b6affb4 | impl 5a891bd | prompts/01_requisitos/R-002_historias_usuario_v1.md</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>commit 2d8efad | impl 71144a5 | prompts/02_diseno/D-003 - Promtp de Diseño FrontEnd (Stich) - v2</t>
+          <t>commit 4568914 | impl 71144a5 | prompts/02_diseno/D-003 - Promtp de Diseño FrontEnd (Stich) - v2</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>commit 21221d4 | impl 5a891bd | prompts/02_diseno/D-003 - Promtp de Diseño FrontEnd (Stich) - v2</t>
+          <t>commit ac826f7 | impl 5a891bd | prompts/02_diseno/D-003 - Promtp de Diseño FrontEnd (Stich) - v2</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>commit af7ce42 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
+          <t>commit 251f9a5 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>commit 61832f7 | impl 5a891bd | prompts/01_requisitos/R-002_historias_usuario_v1.md</t>
+          <t>commit ea3e62a | impl 5a891bd | prompts/01_requisitos/R-002_historias_usuario_v1.md</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>commit 0cfae15 | impl 71144a5 | prompts/01_requisitos/R-002_historias_usuario_v1.md</t>
+          <t>commit 7b17b7b | impl 71144a5 | prompts/01_requisitos/R-002_historias_usuario_v1.md</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2753,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>commit a77b6bb | impl 5a891bd | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
+          <t>commit c0a0952 | impl 5a891bd | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
         </is>
       </c>
     </row>
@@ -2795,7 +2795,7 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>commit f96c2f6 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
+          <t>commit ce43d09 | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
         </is>
       </c>
     </row>
@@ -2837,7 +2837,7 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>commit 1f2f8ce | impl 71144a5 | prompts/01_requisitos/R-002_historias_usuario_v1.md</t>
+          <t>commit 1f31467 | impl 71144a5 | prompts/01_requisitos/R-002_historias_usuario_v1.md</t>
         </is>
       </c>
     </row>
@@ -2879,7 +2879,7 @@
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>commit 6924a69 | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
+          <t>commit 09b175e | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
         </is>
       </c>
     </row>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>commit 65a0cb3 | impl 5a891bd | prompts/02_diseno/D-003 - Promtp de Diseño FrontEnd (Stich) - v2</t>
+          <t>commit 3310b73 | impl 5a891bd | prompts/02_diseno/D-003 - Promtp de Diseño FrontEnd (Stich) - v2</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>commit 425c4fe | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
+          <t>commit b185b2d | impl 5a891bd | prompts/02_diseno/D-001_modelo_datos_v1.md</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3005,7 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>commit dc3da3e | impl 71144a5 | prompts/02_diseno/D-003 - Promtp de Diseño FrontEnd (Stich) - v2</t>
+          <t>commit 60767bd | impl 71144a5 | prompts/02_diseno/D-003 - Promtp de Diseño FrontEnd (Stich) - v2</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>commit 6ef1cdd | impl 71144a5 | prompts/02_diseno/D-003 - Promtp de Diseño FrontEnd (Stich) - v2</t>
+          <t>commit db3e558 | impl 71144a5 | prompts/02_diseno/D-003 - Promtp de Diseño FrontEnd (Stich) - v2</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>commit 7c6a056 | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
+          <t>commit 086a1e5 | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>commit 7677c89 | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
+          <t>commit 54960ad | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3173,7 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>commit 201a1c8 | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
+          <t>commit 1bc52f7 | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
         </is>
       </c>
     </row>
@@ -3215,7 +3215,7 @@
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>commit 636635d | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
+          <t>commit e99962c | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>commit c843789 | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
+          <t>commit 46426ab | impl 71144a5 | prompts/02_diseno/D-002_decision_arquitectura_v1.md</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>commit 3a86b19</t>
+          <t>commit 04c5fef</t>
         </is>
       </c>
       <c r="J2" s="7" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>commit c87eb90</t>
+          <t>commit 8836ddb</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>commit 7d45f96</t>
+          <t>commit 7814d12</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>commit bae1be7</t>
+          <t>commit 1fde769</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>commit c54af96</t>
+          <t>commit f8e9e43</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>commit ca8984c</t>
+          <t>commit 1846117</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>commit aef66a6</t>
+          <t>commit 9406618</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>commit af753d9</t>
+          <t>commit b6affb4</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>commit 2d8efad</t>
+          <t>commit 4568914</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>commit 21221d4</t>
+          <t>commit ac826f7</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
@@ -3902,7 +3902,7 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>commit af7ce42</t>
+          <t>commit 251f9a5</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>commit 61832f7</t>
+          <t>commit ea3e62a</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>commit 0cfae15</t>
+          <t>commit 7b17b7b</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>commit a77b6bb</t>
+          <t>commit c0a0952</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>commit f96c2f6</t>
+          <t>commit ce43d09</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>commit 1f2f8ce</t>
+          <t>commit 1f31467</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>commit 6924a69</t>
+          <t>commit 09b175e</t>
         </is>
       </c>
       <c r="J18" s="7" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>commit 65a0cb3</t>
+          <t>commit 3310b73</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>commit 425c4fe</t>
+          <t>commit b185b2d</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>commit dc3da3e</t>
+          <t>commit 60767bd</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>commit 6ef1cdd</t>
+          <t>commit db3e558</t>
         </is>
       </c>
       <c r="J22" s="7" t="inlineStr">
@@ -4474,7 +4474,7 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>commit 7c6a056</t>
+          <t>commit 086a1e5</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
@@ -4526,7 +4526,7 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>commit 7677c89</t>
+          <t>commit 54960ad</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>commit 201a1c8</t>
+          <t>commit 1bc52f7</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>commit 636635d</t>
+          <t>commit e99962c</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>commit c843789</t>
+          <t>commit 46426ab</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">

</xml_diff>